<commit_message>
Reducir tiempo de carga de los tableros y estandarizar avisos
</commit_message>
<xml_diff>
--- a/data/ArchivosLimpios/new_ruteo.xlsx
+++ b/data/ArchivosLimpios/new_ruteo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,31 @@
           <t>Distancia de Ruta</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cumplimiento Salida (06:30:00)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>% Utilizacion</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>% Visitas Plan</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>% Visitas Clientes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Total Kilos</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -441,6 +466,19 @@
       <c r="C2" t="n">
         <v>4381</v>
       </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -454,6 +492,19 @@
       <c r="C3" t="n">
         <v>69138.89999999999</v>
       </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -467,6 +518,19 @@
       <c r="C4" t="n">
         <v>1895107.2</v>
       </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -480,6 +544,19 @@
       <c r="C5" t="n">
         <v>589540.9</v>
       </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -493,6 +570,19 @@
       <c r="C6" t="n">
         <v>7235.8</v>
       </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -506,6 +596,19 @@
       <c r="C7" t="n">
         <v>83074.89999999999</v>
       </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -519,6 +622,19 @@
       <c r="C8" t="n">
         <v>1498000</v>
       </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -532,6 +648,19 @@
       <c r="C9" t="n">
         <v>14346.6</v>
       </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -545,6 +674,19 @@
       <c r="C10" t="n">
         <v>2187242.3</v>
       </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -558,6 +700,19 @@
       <c r="C11" t="n">
         <v>1969204.4</v>
       </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -571,6 +726,19 @@
       <c r="C12" t="n">
         <v>3853739.4</v>
       </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -584,6 +752,19 @@
       <c r="C13" t="n">
         <v>782066</v>
       </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -597,6 +778,19 @@
       <c r="C14" t="n">
         <v>54091.4</v>
       </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -610,6 +804,19 @@
       <c r="C15" t="n">
         <v>21154.3</v>
       </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -623,6 +830,19 @@
       <c r="C16" t="n">
         <v>45722.5</v>
       </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -636,6 +856,19 @@
       <c r="C17" t="n">
         <v>0</v>
       </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -649,6 +882,19 @@
       <c r="C18" t="n">
         <v>1729509.4</v>
       </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -662,6 +908,19 @@
       <c r="C19" t="n">
         <v>33337.2</v>
       </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -675,6 +934,19 @@
       <c r="C20" t="n">
         <v>15334.6</v>
       </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -688,6 +960,19 @@
       <c r="C21" t="n">
         <v>1484068.8</v>
       </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -701,6 +986,19 @@
       <c r="C22" t="n">
         <v>16761.2</v>
       </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -714,6 +1012,19 @@
       <c r="C23" t="n">
         <v>33864</v>
       </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -727,6 +1038,19 @@
       <c r="C24" t="n">
         <v>99062.8</v>
       </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -740,6 +1064,19 @@
       <c r="C25" t="n">
         <v>4595824.8</v>
       </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -753,6 +1090,19 @@
       <c r="C26" t="n">
         <v>29918.5</v>
       </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -766,6 +1116,19 @@
       <c r="C27" t="n">
         <v>314214.2</v>
       </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -779,6 +1142,19 @@
       <c r="C28" t="n">
         <v>27743.2</v>
       </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -792,6 +1168,19 @@
       <c r="C29" t="n">
         <v>30531.3</v>
       </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -805,6 +1194,19 @@
       <c r="C30" t="n">
         <v>29354.1</v>
       </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -818,6 +1220,19 @@
       <c r="C31" t="n">
         <v>296018.6</v>
       </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -831,6 +1246,19 @@
       <c r="C32" t="n">
         <v>3212162.7</v>
       </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -844,6 +1272,19 @@
       <c r="C33" t="n">
         <v>3854621.3</v>
       </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -857,6 +1298,19 @@
       <c r="C34" t="n">
         <v>5306243.3</v>
       </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -870,6 +1324,19 @@
       <c r="C35" t="n">
         <v>716477.2</v>
       </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -883,6 +1350,19 @@
       <c r="C36" t="n">
         <v>99417.3</v>
       </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>